<commit_message>
done govt multi data can upload
</commit_message>
<xml_diff>
--- a/uploads/govt_plot_excels/govt_(2).xlsx
+++ b/uploads/govt_plot_excels/govt_(2).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maasuser\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{213D0B9A-F878-4C90-99A1-29F1252419D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BBA25F5-18C9-494A-AE71-CBF211BC5B46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="59">
   <si>
     <t>Chendipada</t>
   </si>
@@ -183,6 +183,24 @@
   <si>
     <t>Lease sanctioned by collector</t>
   </si>
+  <si>
+    <t>Dhenkanal</t>
+  </si>
+  <si>
+    <t>Machhagaon</t>
+  </si>
+  <si>
+    <t>Nauga</t>
+  </si>
+  <si>
+    <t>bastijogysa</t>
+  </si>
+  <si>
+    <t>Rajaa</t>
+  </si>
+  <si>
+    <t>100/2009</t>
+  </si>
 </sst>
 </file>
 
@@ -246,7 +264,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -268,9 +286,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -731,7 +746,7 @@
       <c r="H2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="I2" s="9">
+      <c r="I2" s="2">
         <v>142</v>
       </c>
       <c r="J2" s="7">
@@ -820,7 +835,7 @@
       <c r="H3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="I3" s="9">
+      <c r="I3" s="2">
         <v>174</v>
       </c>
       <c r="J3" s="7">
@@ -909,7 +924,7 @@
       <c r="H4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="I4" s="9">
+      <c r="I4" s="2">
         <v>179</v>
       </c>
       <c r="J4" s="7">
@@ -998,7 +1013,7 @@
       <c r="H5" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="I5" s="9">
+      <c r="I5" s="2">
         <v>182</v>
       </c>
       <c r="J5" s="7">
@@ -1087,7 +1102,7 @@
       <c r="H6" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="I6" s="9">
+      <c r="I6" s="2">
         <v>800</v>
       </c>
       <c r="J6" s="7">
@@ -1176,7 +1191,7 @@
       <c r="H7" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="I7" s="9">
+      <c r="I7" s="2">
         <v>809</v>
       </c>
       <c r="J7" s="7">
@@ -1265,7 +1280,7 @@
       <c r="H8" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="I8" s="9">
+      <c r="I8" s="2">
         <v>816</v>
       </c>
       <c r="J8" s="7">
@@ -1329,37 +1344,94 @@
       </c>
       <c r="AE8" s="2"/>
     </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="1"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
-      <c r="L9" s="3"/>
-      <c r="M9" s="3"/>
-      <c r="N9" s="3"/>
-      <c r="O9" s="3"/>
-      <c r="P9" s="3"/>
-      <c r="Q9" s="3"/>
-      <c r="R9" s="3"/>
-      <c r="S9" s="3"/>
-      <c r="T9" s="3"/>
-      <c r="U9" s="3"/>
-      <c r="V9" s="3"/>
-      <c r="W9" s="3"/>
-      <c r="X9" s="3"/>
-      <c r="Y9" s="3"/>
-      <c r="Z9" s="3"/>
-      <c r="AA9" s="3"/>
-      <c r="AB9" s="3"/>
-      <c r="AC9" s="3"/>
-      <c r="AD9" s="3"/>
+    <row r="9" spans="1:31" ht="60" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D9" s="2">
+        <v>42</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="F9" s="5">
+        <v>204</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="I9" s="2">
+        <v>790</v>
+      </c>
+      <c r="J9" s="7">
+        <f t="shared" ref="J9" si="2">L9/2.471</f>
+        <v>1.2545528126264669E-2</v>
+      </c>
+      <c r="K9" s="7">
+        <f t="shared" ref="K9" si="3">M9/2.471</f>
+        <v>1.2545528126264669E-2</v>
+      </c>
+      <c r="L9" s="8">
+        <v>3.1E-2</v>
+      </c>
+      <c r="M9" s="8">
+        <v>3.1E-2</v>
+      </c>
+      <c r="N9" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="O9" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="P9" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q9" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="R9" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="S9" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="T9" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="U9" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="V9" s="2"/>
+      <c r="W9" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="X9" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="Y9" s="2"/>
+      <c r="Z9" s="2"/>
+      <c r="AA9" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AB9" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AC9" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="AD9" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="AE9" s="2"/>
     </row>
     <row r="10" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A10" s="3"/>
@@ -7026,7 +7098,7 @@
       <c r="AD186" s="3"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I9:I1048576">
+  <conditionalFormatting sqref="I10:I1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>